<commit_message>
Fix:Updated DriverFactory to handle headless testing in CI and updated Testclasses to use dataproviders
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="CheckoutData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+  <si>
+    <t xml:space="preserve">UserName </t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
   <si>
     <t>First Name</t>
   </si>
@@ -39,31 +45,25 @@
     <t>Zip/Postal Code</t>
   </si>
   <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
     <t>Ranjitha</t>
   </si>
   <si>
     <t>Kannan</t>
   </si>
   <si>
+    <t>visual_user</t>
+  </si>
+  <si>
     <t>Manoj</t>
   </si>
   <si>
     <t>Kumar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UserName </t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>standard_user</t>
-  </si>
-  <si>
-    <t>secret_sauce</t>
-  </si>
-  <si>
-    <t>visual_user</t>
   </si>
 </sst>
 </file>
@@ -1240,44 +1240,64 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="12.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="14.2222222222222" customWidth="1"/>
-    <col min="3" max="3" width="19.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="17.3333333333333" customWidth="1"/>
+    <col min="2" max="2" width="20.1111111111111" customWidth="1"/>
+    <col min="3" max="3" width="12.7777777777778" customWidth="1"/>
+    <col min="4" max="4" width="14.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="19.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3">
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3">
         <v>12345</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3">
         <v>23456</v>
       </c>
     </row>
@@ -1299,26 +1319,26 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>